<commit_message>
Update historical price analysis 2026-03
</commit_message>
<xml_diff>
--- a/outputs/NSW_historical_prices.xlsx
+++ b/outputs/NSW_historical_prices.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Monthly Data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Heatmap" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Update historical price analysis 2026-04
</commit_message>
<xml_diff>
--- a/outputs/NSW_historical_prices.xlsx
+++ b/outputs/NSW_historical_prices.xlsx
@@ -528,16 +528,16 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>100.02</v>
+        <v>96.7</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>120.42</v>
+        <v>116.51</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>101.14</v>
+        <v>97.61</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>121.93</v>
+        <v>117.8</v>
       </c>
     </row>
     <row r="6">
@@ -547,16 +547,16 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>115.48</v>
+        <v>114.41</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>145.2</v>
+        <v>144.12</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>118.56</v>
+        <v>117.31</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>149.25</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7">
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>107.9</v>
+        <v>106.61</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>132.05</v>
+        <v>130.5</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>112.14</v>
+        <v>110.58</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>137.24</v>
+        <v>135.4</v>
       </c>
     </row>
     <row r="8">
@@ -585,16 +585,16 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>118.8</v>
+        <v>118.94</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>141</v>
+        <v>140.86</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>129.63</v>
+        <v>129.57</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>153.81</v>
+        <v>153.42</v>
       </c>
     </row>
     <row r="9">
@@ -604,22 +604,22 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>97.47</v>
+        <v>97.45999999999999</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>115.39</v>
+        <v>115.24</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>113.49</v>
+        <v>113.29</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>134.31</v>
+        <v>133.95</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Data through: Mar 2026</t>
+          <t>Data through: Apr 2026</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F274"/>
+  <dimension ref="A1:F275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6233,6 +6233,26 @@
       </c>
       <c r="F274" s="7" t="inlineStr"/>
     </row>
+    <row r="275">
+      <c r="A275" s="4" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="B275" s="5" t="n">
+        <v>64.27</v>
+      </c>
+      <c r="C275" s="5" t="n">
+        <v>60.42</v>
+      </c>
+      <c r="D275" s="5" t="n">
+        <v>64.27</v>
+      </c>
+      <c r="E275" s="5" t="n">
+        <v>60.42</v>
+      </c>
+      <c r="F275" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6244,7 +6264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E274"/>
+  <dimension ref="A1:E275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11468,8 +11488,27 @@
         <v>74.36</v>
       </c>
     </row>
+    <row r="275">
+      <c r="A275" s="4" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="B275" s="5" t="n">
+        <v>64.27</v>
+      </c>
+      <c r="C275" s="5" t="n">
+        <v>60.42</v>
+      </c>
+      <c r="D275" s="5" t="n">
+        <v>64.27</v>
+      </c>
+      <c r="E275" s="5" t="n">
+        <v>60.42</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B274">
+  <conditionalFormatting sqref="B2:B275">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -11481,7 +11520,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C274">
+  <conditionalFormatting sqref="C2:C275">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -11493,7 +11532,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D274">
+  <conditionalFormatting sqref="D2:D275">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -11505,7 +11544,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E274">
+  <conditionalFormatting sqref="E2:E275">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
Update historical price analysis 2026-06
</commit_message>
<xml_diff>
--- a/outputs/NSW_historical_prices.xlsx
+++ b/outputs/NSW_historical_prices.xlsx
@@ -528,16 +528,16 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>91.93000000000001</v>
+        <v>76.3</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>108.26</v>
+        <v>77.53</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>93.56999999999999</v>
+        <v>77.23</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>110.44</v>
+        <v>78.51000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -547,16 +547,16 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>105.75</v>
+        <v>102.25</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>128.84</v>
+        <v>124.36</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>109.48</v>
+        <v>105.62</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>133.58</v>
+        <v>128.71</v>
       </c>
     </row>
     <row r="7">
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>103.05</v>
+        <v>102.03</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>125.85</v>
+        <v>124.26</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>107.93</v>
+        <v>106.63</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>131.91</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8">
@@ -585,16 +585,16 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>118.07</v>
+        <v>116.55</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>138.86</v>
+        <v>135.72</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>129.98</v>
+        <v>127.83</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>152.75</v>
+        <v>148.62</v>
       </c>
     </row>
     <row r="9">
@@ -604,22 +604,22 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>97.45</v>
+        <v>97.2</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>115.09</v>
+        <v>114.63</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>114.63</v>
+        <v>114.1</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>135.38</v>
+        <v>134.56</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Data through: May 2026</t>
+          <t>Data through: Jun 2026</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F276"/>
+  <dimension ref="A1:F277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6273,6 +6273,26 @@
       </c>
       <c r="F276" s="7" t="inlineStr"/>
     </row>
+    <row r="277">
+      <c r="A277" s="4" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="B277" s="5" t="n">
+        <v>68.61</v>
+      </c>
+      <c r="C277" s="5" t="n">
+        <v>66.68000000000001</v>
+      </c>
+      <c r="D277" s="5" t="n">
+        <v>68.61</v>
+      </c>
+      <c r="E277" s="5" t="n">
+        <v>66.68000000000001</v>
+      </c>
+      <c r="F277" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6284,7 +6304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E276"/>
+  <dimension ref="A1:E277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11546,8 +11566,27 @@
         <v>63.17</v>
       </c>
     </row>
+    <row r="277">
+      <c r="A277" s="4" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="B277" s="5" t="n">
+        <v>68.61</v>
+      </c>
+      <c r="C277" s="5" t="n">
+        <v>66.68000000000001</v>
+      </c>
+      <c r="D277" s="5" t="n">
+        <v>68.61</v>
+      </c>
+      <c r="E277" s="5" t="n">
+        <v>66.68000000000001</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B276">
+  <conditionalFormatting sqref="B2:B277">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -11559,7 +11598,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C276">
+  <conditionalFormatting sqref="C2:C277">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -11571,7 +11610,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D276">
+  <conditionalFormatting sqref="D2:D277">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -11583,7 +11622,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E276">
+  <conditionalFormatting sqref="E2:E277">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
Update historical price analysis 2026-07
</commit_message>
<xml_diff>
--- a/outputs/NSW_historical_prices.xlsx
+++ b/outputs/NSW_historical_prices.xlsx
@@ -528,16 +528,16 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>76.3</v>
+        <v>74.84</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>77.53</v>
+        <v>75.72</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>77.23</v>
+        <v>75.54000000000001</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>78.51000000000001</v>
+        <v>76.44</v>
       </c>
     </row>
     <row r="6">
@@ -547,16 +547,16 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>102.25</v>
+        <v>100.26</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>124.36</v>
+        <v>121.45</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>105.62</v>
+        <v>103.35</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>128.71</v>
+        <v>125.44</v>
       </c>
     </row>
     <row r="7">
@@ -566,16 +566,16 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>102.03</v>
+        <v>101.9</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>124.26</v>
+        <v>124.04</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>106.63</v>
+        <v>106.29</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>130</v>
+        <v>129.53</v>
       </c>
     </row>
     <row r="8">
@@ -585,16 +585,16 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>116.55</v>
+        <v>115.81</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>135.72</v>
+        <v>134.25</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>127.83</v>
+        <v>126.61</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>148.62</v>
+        <v>146.48</v>
       </c>
     </row>
     <row r="9">
@@ -604,22 +604,22 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>97.2</v>
+        <v>97.31999999999999</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>114.63</v>
+        <v>114.62</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>114.1</v>
+        <v>114.02</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>134.56</v>
+        <v>134.31</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Data through: Jun 2026</t>
+          <t>Data through: Jul 2026</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F277"/>
+  <dimension ref="A1:F278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6293,6 +6293,26 @@
       </c>
       <c r="F277" s="7" t="inlineStr"/>
     </row>
+    <row r="278">
+      <c r="A278" s="4" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="B278" s="5" t="n">
+        <v>79.43000000000001</v>
+      </c>
+      <c r="C278" s="5" t="n">
+        <v>85.61</v>
+      </c>
+      <c r="D278" s="5" t="n">
+        <v>79.43000000000001</v>
+      </c>
+      <c r="E278" s="5" t="n">
+        <v>85.61</v>
+      </c>
+      <c r="F278" s="7" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6304,7 +6324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E277"/>
+  <dimension ref="A1:E278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11585,8 +11605,27 @@
         <v>66.68000000000001</v>
       </c>
     </row>
+    <row r="278">
+      <c r="A278" s="4" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="B278" s="5" t="n">
+        <v>79.43000000000001</v>
+      </c>
+      <c r="C278" s="5" t="n">
+        <v>85.61</v>
+      </c>
+      <c r="D278" s="5" t="n">
+        <v>79.43000000000001</v>
+      </c>
+      <c r="E278" s="5" t="n">
+        <v>85.61</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B277">
+  <conditionalFormatting sqref="B2:B278">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -11598,7 +11637,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C277">
+  <conditionalFormatting sqref="C2:C278">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -11610,7 +11649,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D277">
+  <conditionalFormatting sqref="D2:D278">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -11622,7 +11661,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E277">
+  <conditionalFormatting sqref="E2:E278">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>